<commit_message>
add figures and commit local files, update readme, remove old files
</commit_message>
<xml_diff>
--- a/lit_review_results/2-screening_phase/backward_forward_search.xlsx
+++ b/lit_review_results/2-screening_phase/backward_forward_search.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfrieder/PycharmProjects/sok_artifacts/lit_review_results/2-screening_phase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66245002-8FD9-2546-857C-0531BE8F4CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63CC8C09-281C-884D-8BD9-3AB2A3145BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16620" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7680" yWindow="-28240" windowWidth="51080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="242">
   <si>
     <t>Database</t>
   </si>
@@ -787,6 +787,27 @@
   </si>
   <si>
     <t>check appendix, only referrer and cookie privacy related</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/10850137</t>
+  </si>
+  <si>
+    <t>10.1109/IPCCC59868.2024.10850137</t>
+  </si>
+  <si>
+    <t>Yuan, Yong and Wei, Ziling and Liu, Lin and Chen, Shuhui and Su, Jinshu</t>
+  </si>
+  <si>
+    <t>IPCCC</t>
+  </si>
+  <si>
+    <t>AST-Trans: Detecting Web Tracking using Transformer-based Deep Learning with Abstract Syntax Tree</t>
+  </si>
+  <si>
+    <t>Web tracking has become a key tool for service providers to collect online data and analyze user behaviors, raising concerns about the privacy of Internet users. In this paper, we propose a new web tracking detection method, namely AST-Trans, which detects and removes web tracking behavior using Transformer-based deep learning with abstract syntax trees. In the method, the abstract syntax tree is built for the detected website codes. Then, a sequence generation algorithm is proposed to convert tree-like code structures into one-dimensional sequences for deep models. To enhance training efficiency, we devise a reduction strategy to simplify the code tree structure by introducing equivalent nodes. After that, a Transformer-based deep learning algorithm is introduced to realize web tracking detection. By the proposed method, the exact tracking code blocks can be identified, and thus, we can implement the tracking code removal with minimum website breakage. To verify the effectiveness of the proposed method, an HTTPS proxy with AST-Trans on it is implemented to detect and remove tracking codes. We evaluate AST-Trans with the TrackSign-labeled dataset. The results show that the proposed method can detect the tracking behavior with high precision. In addition, we validate the feasibility of the method by measuring the website page breakage.</t>
+  </si>
+  <si>
+    <t>Web Tracking, Abstract Syntax Tree, Deep learning, Transformer</t>
   </si>
 </sst>
 </file>
@@ -1160,7 +1181,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1222,9 +1243,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1336,12 +1354,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1671,7 +1684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W38"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" style="1" bestFit="1" customWidth="1"/>
@@ -1718,35 +1731,35 @@
       <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="K1" s="25" t="s">
         <v>221</v>
       </c>
-      <c r="L1" s="27" t="s">
+      <c r="L1" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="27" t="s">
+      <c r="M1" s="26" t="s">
         <v>223</v>
       </c>
-      <c r="N1" s="27" t="s">
+      <c r="N1" s="26" t="s">
         <v>224</v>
       </c>
-      <c r="O1" s="28" t="s">
+      <c r="O1" s="27" t="s">
         <v>225</v>
       </c>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="30" t="s">
+      <c r="P1" s="28"/>
+      <c r="Q1" s="29" t="s">
         <v>226</v>
       </c>
-      <c r="R1" s="31" t="s">
+      <c r="R1" s="30" t="s">
         <v>227</v>
       </c>
-      <c r="S1" s="31" t="s">
+      <c r="S1" s="30" t="s">
         <v>228</v>
       </c>
-      <c r="T1" s="31" t="s">
+      <c r="T1" s="30" t="s">
         <v>229</v>
       </c>
-      <c r="U1" s="32" t="s">
+      <c r="U1" s="31" t="s">
         <v>230</v>
       </c>
     </row>
@@ -1777,35 +1790,35 @@
         <v>69</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O2" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S2" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U2" s="39" t="b">
+      <c r="K2" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T2" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1840,88 +1853,88 @@
       <c r="J3" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="K3" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O3" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S3" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U3" s="39" t="b">
+      <c r="K3" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T3" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" s="38" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="53" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42" t="s">
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="40">
+      <c r="E4" s="39">
         <v>2020</v>
       </c>
-      <c r="F4" s="40" t="s">
+      <c r="F4" s="39" t="s">
         <v>197</v>
       </c>
-      <c r="G4" s="40"/>
-      <c r="H4" s="44" t="s">
+      <c r="G4" s="39"/>
+      <c r="H4" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="45"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="47" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" s="49" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" s="50"/>
-      <c r="Q4" s="51" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="S4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="U4" s="52" t="b">
+      <c r="I4" s="44"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="46" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" s="48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="50" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" s="51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1953,36 +1966,36 @@
       <c r="I5" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="J5" s="54"/>
-      <c r="K5" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O5" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R5" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S5" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" s="39" t="b">
+      <c r="J5" s="52"/>
+      <c r="K5" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="35"/>
+      <c r="Q5" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2015,35 +2028,35 @@
         <v>124</v>
       </c>
       <c r="J6" s="13"/>
-      <c r="K6" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N6" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R6" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S6" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U6" s="39" t="b">
+      <c r="K6" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2076,35 +2089,35 @@
         <v>171</v>
       </c>
       <c r="J7" s="13"/>
-      <c r="K7" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" s="36"/>
-      <c r="Q7" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R7" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U7" s="39" t="b">
+      <c r="K7" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" s="35"/>
+      <c r="Q7" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R7" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" s="38" t="b">
         <v>0</v>
       </c>
       <c r="V7" s="1" t="s">
@@ -2142,35 +2155,35 @@
       <c r="J8" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="K8" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M8" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N8" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R8" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S8" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T8" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U8" s="39" t="b">
+      <c r="K8" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P8" s="35"/>
+      <c r="Q8" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R8" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T8" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" s="38" t="b">
         <v>0</v>
       </c>
       <c r="V8" s="1" t="s">
@@ -2211,35 +2224,35 @@
       <c r="J9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="K9" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R9" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S9" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T9" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U9" s="39" t="b">
+      <c r="K9" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S9" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T9" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U9" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2270,35 +2283,35 @@
         <v>158</v>
       </c>
       <c r="J10" s="13"/>
-      <c r="K10" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L10" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M10" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N10" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R10" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T10" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U10" s="39" t="b">
+      <c r="K10" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P10" s="35"/>
+      <c r="Q10" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R10" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S10" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T10" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U10" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2333,35 +2346,35 @@
       <c r="J11" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="K11" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L11" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R11" s="38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S11" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T11" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U11" s="39" t="b">
+      <c r="K11" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T11" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2396,35 +2409,35 @@
       <c r="J12" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="K12" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L12" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M12" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R12" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S12" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T12" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U12" s="39" t="b">
+      <c r="K12" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N12" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="35"/>
+      <c r="Q12" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S12" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T12" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U12" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2459,35 +2472,35 @@
       <c r="J13" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="K13" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L13" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M13" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R13" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S13" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T13" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U13" s="39" t="b">
+      <c r="K13" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N13" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="35"/>
+      <c r="Q13" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S13" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T13" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U13" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2520,35 +2533,35 @@
         <v>180</v>
       </c>
       <c r="J14" s="13"/>
-      <c r="K14" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L14" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M14" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O14" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R14" s="38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S14" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T14" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U14" s="39" t="b">
+      <c r="K14" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N14" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R14" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T14" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U14" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2581,97 +2594,97 @@
         <v>157</v>
       </c>
       <c r="J15" s="13"/>
-      <c r="K15" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L15" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M15" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P15" s="36"/>
-      <c r="Q15" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R15" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T15" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U15" s="39" t="b">
+      <c r="K15" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S15" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T15" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U15" s="38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:23" s="43" customFormat="1" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="40" t="s">
+    <row r="16" spans="1:23" s="42" customFormat="1" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42" t="s">
+      <c r="C16" s="41"/>
+      <c r="D16" s="41" t="s">
         <v>214</v>
       </c>
-      <c r="E16" s="40">
+      <c r="E16" s="39">
         <v>2002</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="F16" s="39" t="s">
         <v>212</v>
       </c>
-      <c r="G16" s="40" t="s">
+      <c r="G16" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="I16" s="45" t="s">
+      <c r="I16" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="J16" s="46"/>
-      <c r="K16" s="47" t="b">
-        <v>0</v>
-      </c>
-      <c r="L16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="M16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16" s="49" t="b">
-        <v>0</v>
-      </c>
-      <c r="P16" s="50"/>
-      <c r="Q16" s="51" t="b">
-        <v>0</v>
-      </c>
-      <c r="R16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="S16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="T16" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="U16" s="52" t="b">
-        <v>0</v>
-      </c>
-      <c r="V16" s="43" t="s">
+      <c r="J16" s="45"/>
+      <c r="K16" s="46" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" s="48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="50" t="b">
+        <v>0</v>
+      </c>
+      <c r="R16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="S16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="U16" s="51" t="b">
+        <v>0</v>
+      </c>
+      <c r="V16" s="42" t="s">
         <v>232</v>
       </c>
     </row>
@@ -2706,35 +2719,35 @@
       <c r="J17" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="K17" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L17" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O17" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P17" s="36"/>
-      <c r="Q17" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R17" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S17" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T17" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U17" s="39" t="b">
+      <c r="K17" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P17" s="35"/>
+      <c r="Q17" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R17" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S17" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T17" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U17" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2767,35 +2780,35 @@
         <v>203</v>
       </c>
       <c r="J18" s="13"/>
-      <c r="K18" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L18" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M18" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N18" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R18" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S18" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T18" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U18" s="39" t="b">
+      <c r="K18" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N18" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O18" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P18" s="35"/>
+      <c r="Q18" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R18" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T18" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U18" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2828,35 +2841,35 @@
         <v>193</v>
       </c>
       <c r="J19" s="13"/>
-      <c r="K19" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L19" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M19" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N19" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O19" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R19" s="38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S19" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T19" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U19" s="39" t="b">
+      <c r="K19" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M19" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N19" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T19" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U19" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2889,35 +2902,35 @@
         <v>86</v>
       </c>
       <c r="J20" s="13"/>
-      <c r="K20" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L20" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M20" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N20" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R20" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S20" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T20" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U20" s="39" t="b">
+      <c r="K20" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S20" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T20" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U20" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2950,35 +2963,35 @@
         <v>218</v>
       </c>
       <c r="J21" s="13"/>
-      <c r="K21" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L21" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M21" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O21" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R21" s="38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S21" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T21" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U21" s="39" t="b">
+      <c r="K21" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M21" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N21" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O21" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T21" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U21" s="38" t="b">
         <v>0</v>
       </c>
       <c r="V21" s="1" t="s">
@@ -3012,35 +3025,35 @@
         <v>105</v>
       </c>
       <c r="J22" s="13"/>
-      <c r="K22" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L22" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M22" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N22" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O22" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P22" s="36"/>
-      <c r="Q22" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R22" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S22" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T22" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U22" s="39" t="b">
+      <c r="K22" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S22" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T22" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U22" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3073,35 +3086,35 @@
         <v>130</v>
       </c>
       <c r="J23" s="13"/>
-      <c r="K23" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L23" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M23" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O23" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P23" s="36"/>
-      <c r="Q23" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R23" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S23" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T23" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U23" s="39" t="b">
+      <c r="K23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M23" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P23" s="35"/>
+      <c r="Q23" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R23" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S23" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T23" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U23" s="38" t="b">
         <v>0</v>
       </c>
       <c r="V23" s="1" t="s">
@@ -3139,35 +3152,35 @@
       <c r="J24" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="K24" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L24" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M24" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N24" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R24" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S24" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T24" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U24" s="39" t="b">
+      <c r="K24" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P24" s="35"/>
+      <c r="Q24" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R24" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S24" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T24" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U24" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3202,90 +3215,93 @@
       <c r="J25" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="K25" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M25" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O25" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P25" s="36"/>
-      <c r="Q25" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R25" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S25" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T25" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U25" s="39" t="b">
-        <v>0</v>
+      <c r="K25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P25" s="35"/>
+      <c r="Q25" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R25" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S25" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U25" s="38" t="b">
+        <v>0</v>
+      </c>
+      <c r="V25" s="1" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42" t="s">
+      <c r="C26" s="41"/>
+      <c r="D26" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="40">
+      <c r="E26" s="39">
         <v>2022</v>
       </c>
-      <c r="F26" s="40" t="s">
+      <c r="F26" s="39" t="s">
         <v>197</v>
       </c>
-      <c r="G26" s="40"/>
-      <c r="H26" s="44" t="s">
+      <c r="G26" s="39"/>
+      <c r="H26" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="I26" s="45"/>
-      <c r="J26" s="46"/>
-      <c r="K26" s="47" t="b">
-        <v>0</v>
-      </c>
-      <c r="L26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="M26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="N26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="O26" s="49" t="b">
-        <v>0</v>
-      </c>
-      <c r="P26" s="50"/>
-      <c r="Q26" s="51" t="b">
-        <v>0</v>
-      </c>
-      <c r="R26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="S26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="T26" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="U26" s="52" t="b">
+      <c r="I26" s="44"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="46" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="N26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" s="48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" s="49"/>
+      <c r="Q26" s="50" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="S26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T26" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="U26" s="51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3302,13 +3318,13 @@
       <c r="D27" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E27" s="53">
+      <c r="E27" s="1">
         <v>2020</v>
       </c>
-      <c r="F27" s="23" t="s">
+      <c r="F27" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="G27" s="53" t="s">
+      <c r="G27" s="1" t="s">
         <v>64</v>
       </c>
       <c r="H27" s="11" t="s">
@@ -3317,36 +3333,36 @@
       <c r="I27" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="J27" s="55"/>
-      <c r="K27" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L27" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M27" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N27" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O27" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P27" s="36"/>
-      <c r="Q27" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R27" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S27" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T27" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U27" s="39" t="b">
+      <c r="J27" s="15"/>
+      <c r="K27" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M27" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N27" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O27" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S27" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T27" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U27" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3381,35 +3397,35 @@
       <c r="J28" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="K28" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L28" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M28" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N28" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P28" s="36"/>
-      <c r="Q28" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R28" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S28" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T28" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U28" s="39" t="b">
+      <c r="K28" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M28" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N28" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O28" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R28" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T28" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U28" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3440,39 +3456,39 @@
         <v>190</v>
       </c>
       <c r="J29" s="13"/>
-      <c r="K29" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L29" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M29" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N29" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O29" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P29" s="36"/>
-      <c r="Q29" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R29" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S29" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T29" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U29" s="39" t="b">
+      <c r="K29" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M29" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N29" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O29" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P29" s="35"/>
+      <c r="Q29" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S29" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T29" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U29" s="38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:22" s="56" customFormat="1" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" ht="138" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
@@ -3501,35 +3517,35 @@
         <v>73</v>
       </c>
       <c r="J30" s="13"/>
-      <c r="K30" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L30" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M30" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N30" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O30" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P30" s="36"/>
-      <c r="Q30" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R30" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S30" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T30" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U30" s="39" t="b">
+      <c r="K30" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M30" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N30" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O30" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R30" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S30" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T30" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U30" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3564,35 +3580,35 @@
       <c r="J31" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="K31" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L31" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M31" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N31" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O31" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P31" s="36"/>
-      <c r="Q31" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R31" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S31" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T31" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U31" s="39" t="b">
+      <c r="K31" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M31" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N31" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O31" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R31" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S31" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T31" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U31" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3625,35 +3641,35 @@
         <v>166</v>
       </c>
       <c r="J32" s="13"/>
-      <c r="K32" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L32" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M32" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N32" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O32" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P32" s="36"/>
-      <c r="Q32" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R32" s="38" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T32" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U32" s="39" t="b">
+      <c r="K32" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M32" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N32" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P32" s="35"/>
+      <c r="Q32" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R32" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T32" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U32" s="38" t="b">
         <v>0</v>
       </c>
       <c r="V32" s="1" t="s">
@@ -3691,39 +3707,39 @@
       <c r="J33" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="K33" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L33" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M33" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N33" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O33" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P33" s="36"/>
-      <c r="Q33" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R33" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S33" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T33" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U33" s="39" t="b">
+      <c r="K33" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L33" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M33" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N33" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O33" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P33" s="35"/>
+      <c r="Q33" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R33" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S33" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T33" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U33" s="38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:21" s="56" customFormat="1" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>61</v>
       </c>
@@ -3742,7 +3758,7 @@
       <c r="F34" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G34" s="53" t="s">
+      <c r="G34" s="1" t="s">
         <v>82</v>
       </c>
       <c r="H34" s="11" t="s">
@@ -3754,35 +3770,35 @@
       <c r="J34" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="K34" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L34" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M34" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N34" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O34" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P34" s="36"/>
-      <c r="Q34" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R34" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S34" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T34" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U34" s="39" t="b">
+      <c r="K34" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L34" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M34" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N34" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O34" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P34" s="35"/>
+      <c r="Q34" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R34" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S34" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T34" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U34" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3815,35 +3831,35 @@
         <v>215</v>
       </c>
       <c r="J35" s="13"/>
-      <c r="K35" s="33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L35" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M35" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N35" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O35" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P35" s="36"/>
-      <c r="Q35" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="R35" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S35" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T35" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U35" s="39" t="b">
+      <c r="K35" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L35" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M35" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N35" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O35" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P35" s="35"/>
+      <c r="Q35" s="36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S35" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T35" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U35" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3867,42 +3883,42 @@
       <c r="G36" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H36" s="24" t="s">
+      <c r="H36" s="23" t="s">
         <v>19</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>109</v>
       </c>
       <c r="J36" s="13"/>
-      <c r="K36" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L36" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M36" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N36" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O36" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P36" s="36"/>
-      <c r="Q36" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R36" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S36" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T36" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U36" s="39" t="b">
+      <c r="K36" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L36" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M36" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N36" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O36" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P36" s="35"/>
+      <c r="Q36" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R36" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S36" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T36" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U36" s="38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3928,7 +3944,7 @@
       <c r="G37" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="25" t="s">
+      <c r="H37" s="24" t="s">
         <v>21</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3937,39 +3953,102 @@
       <c r="J37" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="K37" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L37" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="M37" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N37" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O37" s="35" t="b">
-        <v>1</v>
-      </c>
-      <c r="P37" s="36"/>
-      <c r="Q37" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="R37" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="S37" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="T37" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="U37" s="39" t="b">
+      <c r="K37" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L37" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M37" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N37" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O37" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P37" s="35"/>
+      <c r="Q37" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R37" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S37" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T37" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U37" s="38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:21" ht="206" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E38" s="2">
+        <v>2024</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H38" s="24" t="s">
+        <v>239</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="K38" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L38" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M38" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="N38" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="O38" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P38" s="35"/>
+      <c r="Q38" s="36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R38" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="S38" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T38" s="37" t="b">
+        <v>0</v>
+      </c>
+      <c r="U38" s="38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <autoFilter ref="A1:U38" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U38">
@@ -3991,25 +4070,25 @@
     <hyperlink ref="B34" r:id="rId11" xr:uid="{DCF7A2EA-5244-5D42-9E91-EFD42074BD83}"/>
     <hyperlink ref="B22" r:id="rId12" xr:uid="{362D804A-DCB0-854C-A0E3-E75F5FE497A7}"/>
     <hyperlink ref="B13" r:id="rId13" xr:uid="{60AFD93A-E10C-824A-A42B-25AD906DCAF7}"/>
-    <hyperlink ref="B37" r:id="rId14" xr:uid="{926644E3-ABA7-C84F-BE16-413D233FB6D0}"/>
-    <hyperlink ref="B6" r:id="rId15" xr:uid="{E316690B-3EDE-ED42-98A4-982A1547AEA3}"/>
-    <hyperlink ref="B23" r:id="rId16" xr:uid="{4D68A812-C2D8-394C-B7CC-8F3AB4681691}"/>
-    <hyperlink ref="B17" r:id="rId17" xr:uid="{FFCA4C7E-2ED7-B741-B06E-0F9AA38FF196}"/>
-    <hyperlink ref="B33" r:id="rId18" xr:uid="{E51E509C-C792-7447-BD90-EFF76F8EB577}"/>
-    <hyperlink ref="B25" r:id="rId19" xr:uid="{D1FAE453-4D75-5A40-9B38-787160156EBA}"/>
-    <hyperlink ref="B10" r:id="rId20" xr:uid="{9B445229-3E8D-E949-96C8-D887F20D6A9F}"/>
-    <hyperlink ref="B28" r:id="rId21" xr:uid="{95DF12B2-FE81-9249-B89A-273E1E374690}"/>
-    <hyperlink ref="B32" r:id="rId22" xr:uid="{30FA1844-DC2C-E744-BD3E-8BE60B5C187A}"/>
-    <hyperlink ref="B7" r:id="rId23" xr:uid="{2C5918E8-0E10-C945-98E8-28C2650916C0}"/>
-    <hyperlink ref="B14" r:id="rId24" xr:uid="{1DEC30E3-E66C-9942-8A3B-C011462547F9}"/>
-    <hyperlink ref="B9" r:id="rId25" xr:uid="{DF3B9494-08D1-3740-B27D-6E5AACDBE799}"/>
-    <hyperlink ref="B29" r:id="rId26" xr:uid="{0F772668-C9B8-B34E-B434-4BB9EFFDEB0B}"/>
-    <hyperlink ref="B18" r:id="rId27" xr:uid="{099D24AD-0849-B242-A129-193C00A45918}"/>
-    <hyperlink ref="B11" r:id="rId28" xr:uid="{C06522C4-A7D7-A94F-B851-CEE27F3853D3}"/>
-    <hyperlink ref="B26" r:id="rId29" xr:uid="{AAC02283-C0C8-FD44-A7DA-453A5187DA6E}"/>
-    <hyperlink ref="B16" r:id="rId30" xr:uid="{71133B5A-1ECA-E34F-92BD-9557E08314A8}"/>
-    <hyperlink ref="B35" r:id="rId31" xr:uid="{81186F30-D310-C44F-9370-C4E968982319}"/>
-    <hyperlink ref="B21" r:id="rId32" location="citations" xr:uid="{7D6046FE-141D-704F-8F2E-3BEC720D45C6}"/>
+    <hyperlink ref="B6" r:id="rId14" xr:uid="{E316690B-3EDE-ED42-98A4-982A1547AEA3}"/>
+    <hyperlink ref="B23" r:id="rId15" xr:uid="{4D68A812-C2D8-394C-B7CC-8F3AB4681691}"/>
+    <hyperlink ref="B17" r:id="rId16" xr:uid="{FFCA4C7E-2ED7-B741-B06E-0F9AA38FF196}"/>
+    <hyperlink ref="B33" r:id="rId17" xr:uid="{E51E509C-C792-7447-BD90-EFF76F8EB577}"/>
+    <hyperlink ref="B25" r:id="rId18" xr:uid="{D1FAE453-4D75-5A40-9B38-787160156EBA}"/>
+    <hyperlink ref="B10" r:id="rId19" xr:uid="{9B445229-3E8D-E949-96C8-D887F20D6A9F}"/>
+    <hyperlink ref="B28" r:id="rId20" xr:uid="{95DF12B2-FE81-9249-B89A-273E1E374690}"/>
+    <hyperlink ref="B32" r:id="rId21" xr:uid="{30FA1844-DC2C-E744-BD3E-8BE60B5C187A}"/>
+    <hyperlink ref="B7" r:id="rId22" xr:uid="{2C5918E8-0E10-C945-98E8-28C2650916C0}"/>
+    <hyperlink ref="B14" r:id="rId23" xr:uid="{1DEC30E3-E66C-9942-8A3B-C011462547F9}"/>
+    <hyperlink ref="B9" r:id="rId24" xr:uid="{DF3B9494-08D1-3740-B27D-6E5AACDBE799}"/>
+    <hyperlink ref="B29" r:id="rId25" xr:uid="{0F772668-C9B8-B34E-B434-4BB9EFFDEB0B}"/>
+    <hyperlink ref="B18" r:id="rId26" xr:uid="{099D24AD-0849-B242-A129-193C00A45918}"/>
+    <hyperlink ref="B11" r:id="rId27" xr:uid="{C06522C4-A7D7-A94F-B851-CEE27F3853D3}"/>
+    <hyperlink ref="B26" r:id="rId28" xr:uid="{AAC02283-C0C8-FD44-A7DA-453A5187DA6E}"/>
+    <hyperlink ref="B16" r:id="rId29" xr:uid="{71133B5A-1ECA-E34F-92BD-9557E08314A8}"/>
+    <hyperlink ref="B35" r:id="rId30" xr:uid="{81186F30-D310-C44F-9370-C4E968982319}"/>
+    <hyperlink ref="B21" r:id="rId31" location="citations" xr:uid="{7D6046FE-141D-704F-8F2E-3BEC720D45C6}"/>
+    <hyperlink ref="B37" r:id="rId32" xr:uid="{926644E3-ABA7-C84F-BE16-413D233FB6D0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>